<commit_message>
data: 补记 2026-08-26 黄金卖出 1.5 克实收 1492 元
- 黄金持仓 31.5 -> 30 克（成本价 966/克 不变）
- 出入金补一笔「取出 1492 · 黄金卖出」，累计已卖出变现 28762 -> 30254
- 净值历史 8/26 起按 30 克重算：黄金市值、总资产、当日盈亏（扣除该笔取现）、累计盈亏
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B103"/>
+  <dimension ref="A1:B106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1737,6 +1737,42 @@
       <c r="B103" t="inlineStr">
         <is>
           <t>修改 现金 可用资金: 数量 38765→50363.79 成本 0→None 金额 38765→50363.79；修改 现金 可用资金: 成本 0→None；修改 股票 半导体设备: 数量 11300→1300 成本 0.982→-0.386</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-09-18 11:01:57</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>修改 股票 立讯精密: 数量 400→500 成本 61.383→59.485；修改 现金 可用资金: 成本 0→None；修改 现金 可用资金: 成本 0→None</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-09-18 11:02:21</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>修改 现金 可用资金: 数量 50363.79→45048.79 成本 0→None 金额 50363.79→45048.79；修改 现金 可用资金: 成本 0→None</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-09-18 11:10:00</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>更正：补记 2026-08-26 黄金卖出 1.5 克实收 1492 元；黄金持仓 31.5→30 克；净值历史 8/26 起按 30 克重算</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1894,7 @@
         <v>168.54</v>
       </c>
       <c r="G2" t="n">
-        <v>169.86</v>
+        <v>170.5</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -1901,19 +1937,19 @@
         <v>38.159</v>
       </c>
       <c r="G3" t="n">
-        <v>35.15</v>
+        <v>35.22</v>
       </c>
       <c r="H3" t="n">
-        <v>28120</v>
+        <v>28176</v>
       </c>
       <c r="I3" t="n">
-        <v>-2407.2</v>
+        <v>-2351.2</v>
       </c>
       <c r="J3" t="n">
-        <v>-0.0789</v>
+        <v>-0.077</v>
       </c>
       <c r="K3" t="n">
-        <v>0.2143</v>
+        <v>0.2056</v>
       </c>
     </row>
     <row r="4">
@@ -1944,19 +1980,19 @@
         <v>53.404</v>
       </c>
       <c r="G4" t="n">
-        <v>44.79</v>
+        <v>44.89</v>
       </c>
       <c r="H4" t="n">
-        <v>22395</v>
+        <v>22445</v>
       </c>
       <c r="I4" t="n">
-        <v>-4307</v>
+        <v>-4257</v>
       </c>
       <c r="J4" t="n">
-        <v>-0.1613</v>
+        <v>-0.1594</v>
       </c>
       <c r="K4" t="n">
-        <v>0.1707</v>
+        <v>0.1638</v>
       </c>
     </row>
     <row r="5">
@@ -1981,25 +2017,25 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="F5" t="n">
-        <v>61.383</v>
+        <v>59.485</v>
       </c>
       <c r="G5" t="n">
-        <v>53.1</v>
+        <v>53.45</v>
       </c>
       <c r="H5" t="n">
-        <v>21240</v>
+        <v>26725</v>
       </c>
       <c r="I5" t="n">
-        <v>-3313.2</v>
+        <v>-3017.5</v>
       </c>
       <c r="J5" t="n">
-        <v>-0.1349</v>
+        <v>-0.1015</v>
       </c>
       <c r="K5" t="n">
-        <v>0.1619</v>
+        <v>0.195</v>
       </c>
     </row>
     <row r="6">
@@ -2030,7 +2066,7 @@
         <v>258.743</v>
       </c>
       <c r="G6" t="n">
-        <v>69.3</v>
+        <v>69.31</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -2078,7 +2114,7 @@
         <v>65.404</v>
       </c>
       <c r="G7" t="n">
-        <v>42.42</v>
+        <v>42.56</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -2110,7 +2146,7 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>50363.79</v>
+        <v>45048.79</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -2119,7 +2155,7 @@
         <v>0</v>
       </c>
       <c r="H8" t="n">
-        <v>50363.79</v>
+        <v>45048.79</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
@@ -2158,22 +2194,22 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>31.5</v>
+        <v>30</v>
       </c>
       <c r="F9" t="n">
         <v>966</v>
       </c>
       <c r="G9" t="n">
-        <v>939.5700000000001</v>
+        <v>939.24</v>
       </c>
       <c r="H9" t="n">
-        <v>29596.46</v>
+        <v>28177.2</v>
       </c>
       <c r="I9" t="n">
-        <v>-832.54</v>
+        <v>-802.8</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.0274</v>
+        <v>-0.0277</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -2207,16 +2243,16 @@
         <v>14.896</v>
       </c>
       <c r="G10" t="n">
-        <v>12.73</v>
+        <v>12.74</v>
       </c>
       <c r="H10" t="n">
-        <v>10184</v>
+        <v>10192</v>
       </c>
       <c r="I10" t="n">
-        <v>-1732.8</v>
+        <v>-1724.8</v>
       </c>
       <c r="J10" t="n">
-        <v>-0.1454</v>
+        <v>-0.1447</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -2298,7 +2334,7 @@
         <v>1.292</v>
       </c>
       <c r="G12" t="n">
-        <v>1.037</v>
+        <v>1.05</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -2341,7 +2377,7 @@
         <v>28.261</v>
       </c>
       <c r="G13" t="n">
-        <v>32.41</v>
+        <v>32.34</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -2384,7 +2420,7 @@
         <v>84.246</v>
       </c>
       <c r="G14" t="n">
-        <v>50.3</v>
+        <v>50.77</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -2427,19 +2463,19 @@
         <v>-0.386</v>
       </c>
       <c r="G15" t="n">
-        <v>1.163</v>
+        <v>1.178</v>
       </c>
       <c r="H15" t="n">
-        <v>1511.9</v>
+        <v>1531.4</v>
       </c>
       <c r="I15" t="n">
-        <v>2013.7</v>
+        <v>2033.2</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0.0115</v>
+        <v>0.0112</v>
       </c>
     </row>
     <row r="16">
@@ -2470,7 +2506,7 @@
         <v>100</v>
       </c>
       <c r="G16" t="n">
-        <v>141.862</v>
+        <v>142.085</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -2513,19 +2549,19 @@
         <v>1.68</v>
       </c>
       <c r="G17" t="n">
-        <v>1.742</v>
+        <v>1.76</v>
       </c>
       <c r="H17" t="n">
-        <v>24388</v>
+        <v>24640</v>
       </c>
       <c r="I17" t="n">
-        <v>868</v>
+        <v>1120</v>
       </c>
       <c r="J17" t="n">
-        <v>0.0369</v>
+        <v>0.0476</v>
       </c>
       <c r="K17" t="n">
-        <v>0.1859</v>
+        <v>0.1798</v>
       </c>
     </row>
     <row r="18">
@@ -2556,19 +2592,19 @@
         <v>117.251</v>
       </c>
       <c r="G18" t="n">
-        <v>111.81</v>
+        <v>111.77</v>
       </c>
       <c r="H18" t="n">
-        <v>33543</v>
+        <v>33531</v>
       </c>
       <c r="I18" t="n">
-        <v>-1632.3</v>
+        <v>-1644.3</v>
       </c>
       <c r="J18" t="n">
-        <v>-0.0464</v>
+        <v>-0.0467</v>
       </c>
       <c r="K18" t="n">
-        <v>0.2557</v>
+        <v>0.2447</v>
       </c>
     </row>
     <row r="19">
@@ -2578,10 +2614,10 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>220769.47</v>
+        <v>222726.97</v>
       </c>
       <c r="I19" t="n">
-        <v>-12635.5</v>
+        <v>-10050.5</v>
       </c>
     </row>
   </sheetData>
@@ -3890,19 +3926,19 @@
         <v>184709.8</v>
       </c>
       <c r="C43" t="n">
-        <v>31698.13</v>
+        <v>30188.7</v>
       </c>
       <c r="D43" t="n">
         <v>10201.68</v>
       </c>
       <c r="E43" t="n">
-        <v>226609.61</v>
+        <v>225100.18</v>
       </c>
       <c r="F43" t="n">
-        <v>853.35</v>
+        <v>835.92</v>
       </c>
       <c r="G43" t="n">
-        <v>-23557.58</v>
+        <v>-23618.01</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -3920,19 +3956,19 @@
         <v>185801.4</v>
       </c>
       <c r="C44" t="n">
-        <v>31456.53</v>
+        <v>29958.6</v>
       </c>
       <c r="D44" t="n">
         <v>10153.68</v>
       </c>
       <c r="E44" t="n">
-        <v>227411.61</v>
+        <v>225913.68</v>
       </c>
       <c r="F44" t="n">
-        <v>802</v>
+        <v>813.5</v>
       </c>
       <c r="G44" t="n">
-        <v>-22762.48</v>
+        <v>-22811.41</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -3950,19 +3986,19 @@
         <v>180054.1</v>
       </c>
       <c r="C45" t="n">
-        <v>30054.15</v>
+        <v>28623</v>
       </c>
       <c r="D45" t="n">
         <v>10497.68</v>
       </c>
       <c r="E45" t="n">
-        <v>220605.93</v>
+        <v>219174.78</v>
       </c>
       <c r="F45" t="n">
-        <v>-6805.68</v>
+        <v>-6738.9</v>
       </c>
       <c r="G45" t="n">
-        <v>-29708.66</v>
+        <v>-29690.81</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -3980,19 +4016,19 @@
         <v>178445.4</v>
       </c>
       <c r="C46" t="n">
-        <v>29673.94</v>
+        <v>28260.9</v>
       </c>
       <c r="D46" t="n">
         <v>10313.68</v>
       </c>
       <c r="E46" t="n">
-        <v>218433.02</v>
+        <v>217019.98</v>
       </c>
       <c r="F46" t="n">
-        <v>-2172.91</v>
+        <v>-2154.8</v>
       </c>
       <c r="G46" t="n">
-        <v>-31881.57</v>
+        <v>-31845.61</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -4010,19 +4046,19 @@
         <v>178974</v>
       </c>
       <c r="C47" t="n">
-        <v>29350.76</v>
+        <v>27953.1</v>
       </c>
       <c r="D47" t="n">
         <v>10353.68</v>
       </c>
       <c r="E47" t="n">
-        <v>218678.44</v>
+        <v>217280.78</v>
       </c>
       <c r="F47" t="n">
-        <v>245.42</v>
+        <v>260.8</v>
       </c>
       <c r="G47" t="n">
-        <v>-31651.95</v>
+        <v>-31600.61</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -4210,7 +4246,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4356,6 +4392,26 @@
         <v>25153</v>
       </c>
       <c r="D7" t="inlineStr">
+        <is>
+          <t>黄金卖出</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-08-26 12:00</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>取出</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1492</v>
+      </c>
+      <c r="D8" t="inlineStr">
         <is>
           <t>黄金卖出</t>
         </is>
@@ -4912,7 +4968,7 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>31.5</v>
+        <v>30</v>
       </c>
       <c r="F9" t="n">
         <v>966</v>

</xml_diff>

<commit_message>
data: 补记 2026-08-21 黄金基金赎回 3317.32 元
按当日上金所 Au99.99 收盘 983.56 元/克折算 3.37 克，黄金克数链
57.5 → 54.13(8/21) → 28.13(8/24) → 26.63(8/26)；净值历史 8/24、
8/25 按 28.13 克、8/26 起按 26.63 克重算总资产/当日盈亏/累计盈亏。

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/portfolio.xlsx
+++ b/portfolio.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B106"/>
+  <dimension ref="A1:B107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1773,6 +1773,18 @@
       <c r="B106" t="inlineStr">
         <is>
           <t>更正：补记 2026-08-26 黄金卖出 1.5 克实收 1492 元；黄金持仓 31.5→30 克；净值历史 8/26 起按 30 克重算</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-09-18 11:48:01</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>更正：补记 2026-08-21 黄金卖出 3317.32 元（黄金基金赎回，按当日 Au99.99 收盘 983.56 元/克折算 3.37 克）；黄金持仓 30→26.63 克；净值历史 8/24、8/25 按 28.13 克、8/26 起按 26.63 克重算</t>
         </is>
       </c>
     </row>
@@ -2194,22 +2206,22 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>30</v>
+        <v>26.63</v>
       </c>
       <c r="F9" t="n">
         <v>966</v>
       </c>
       <c r="G9" t="n">
-        <v>938.42</v>
+        <v>942.38</v>
       </c>
       <c r="H9" t="n">
-        <v>28152.6</v>
+        <v>25095.58</v>
       </c>
       <c r="I9" t="n">
-        <v>-827.4</v>
+        <v>-629</v>
       </c>
       <c r="J9" t="n">
-        <v>-0.0286</v>
+        <v>-0.0245</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -2614,10 +2626,10 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>222726.97</v>
+        <v>219564.49</v>
       </c>
       <c r="I19" t="n">
-        <v>-10050.5</v>
+        <v>-9957.559999999999</v>
       </c>
     </row>
   </sheetData>
@@ -3866,19 +3878,19 @@
         <v>182915.7</v>
       </c>
       <c r="C41" t="n">
-        <v>31685.22</v>
+        <v>28295.4</v>
       </c>
       <c r="D41" t="n">
         <v>9889.68</v>
       </c>
       <c r="E41" t="n">
-        <v>224490.6</v>
+        <v>221100.78</v>
       </c>
       <c r="F41" t="n">
-        <v>941.15</v>
+        <v>868.65</v>
       </c>
       <c r="G41" t="n">
-        <v>-28964.79</v>
+        <v>-29099.19</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -3896,19 +3908,19 @@
         <v>183869.3</v>
       </c>
       <c r="C42" t="n">
-        <v>31661.28</v>
+        <v>28274.03</v>
       </c>
       <c r="D42" t="n">
         <v>10225.68</v>
       </c>
       <c r="E42" t="n">
-        <v>225756.26</v>
+        <v>222369.01</v>
       </c>
       <c r="F42" t="n">
-        <v>1265.66</v>
+        <v>1268.23</v>
       </c>
       <c r="G42" t="n">
-        <v>-24408.43</v>
+        <v>-24540.26</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -3926,19 +3938,19 @@
         <v>184709.8</v>
       </c>
       <c r="C43" t="n">
-        <v>30188.7</v>
+        <v>26797.5</v>
       </c>
       <c r="D43" t="n">
         <v>10201.68</v>
       </c>
       <c r="E43" t="n">
-        <v>225100.18</v>
+        <v>221708.98</v>
       </c>
       <c r="F43" t="n">
-        <v>835.92</v>
+        <v>831.97</v>
       </c>
       <c r="G43" t="n">
-        <v>-23618.01</v>
+        <v>-23753.79</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -3956,19 +3968,19 @@
         <v>185801.4</v>
       </c>
       <c r="C44" t="n">
-        <v>29958.6</v>
+        <v>26593.25</v>
       </c>
       <c r="D44" t="n">
         <v>10153.68</v>
       </c>
       <c r="E44" t="n">
-        <v>225913.68</v>
+        <v>222548.33</v>
       </c>
       <c r="F44" t="n">
-        <v>813.5</v>
+        <v>839.35</v>
       </c>
       <c r="G44" t="n">
-        <v>-22811.41</v>
+        <v>-22921.34</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -3986,19 +3998,19 @@
         <v>180054.1</v>
       </c>
       <c r="C45" t="n">
-        <v>28623</v>
+        <v>25407.68</v>
       </c>
       <c r="D45" t="n">
         <v>10497.68</v>
       </c>
       <c r="E45" t="n">
-        <v>219174.78</v>
+        <v>215959.46</v>
       </c>
       <c r="F45" t="n">
-        <v>-6738.9</v>
+        <v>-6588.87</v>
       </c>
       <c r="G45" t="n">
-        <v>-29690.81</v>
+        <v>-29650.71</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -4016,19 +4028,19 @@
         <v>178445.4</v>
       </c>
       <c r="C46" t="n">
-        <v>28260.9</v>
+        <v>25086.26</v>
       </c>
       <c r="D46" t="n">
         <v>10313.68</v>
       </c>
       <c r="E46" t="n">
-        <v>217019.98</v>
+        <v>213845.34</v>
       </c>
       <c r="F46" t="n">
-        <v>-2154.8</v>
+        <v>-2114.12</v>
       </c>
       <c r="G46" t="n">
-        <v>-31845.61</v>
+        <v>-31764.83</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -4046,19 +4058,19 @@
         <v>178974</v>
       </c>
       <c r="C47" t="n">
-        <v>27953.1</v>
+        <v>24813.04</v>
       </c>
       <c r="D47" t="n">
         <v>10353.68</v>
       </c>
       <c r="E47" t="n">
-        <v>217280.78</v>
+        <v>214140.72</v>
       </c>
       <c r="F47" t="n">
-        <v>260.8</v>
+        <v>295.38</v>
       </c>
       <c r="G47" t="n">
-        <v>-31600.61</v>
+        <v>-31485.25</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -4246,7 +4258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4380,7 +4392,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-08-24 18:22</t>
+          <t>2026-08-21 14:00</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -4389,7 +4401,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>25153</v>
+        <v>3317.32</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -4400,18 +4412,38 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>2026-08-24 18:22</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>取出</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>25153</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>黄金卖出</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>2026-08-26 12:00</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>取出</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="C9" t="n">
         <v>1492</v>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>黄金卖出</t>
         </is>

</xml_diff>